<commit_message>
Cordes : un repère par corde regroupant ses 3-4 voies sur le plan, colonne Corde à l'import
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UfDVjimRQgJU4TKGnZT47C
</commit_message>
<xml_diff>
--- a/modele_voies.xlsx
+++ b/modele_voies.xlsx
@@ -423,14 +423,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -451,10 +452,15 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Corde</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Secteur</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Hauteur</t>
         </is>
@@ -474,12 +480,15 @@
           <t>4a</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>8</v>
       </c>
     </row>
@@ -497,12 +506,15 @@
           <t>4c</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -520,13 +532,16 @@
           <t>5b</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>10</v>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -535,21 +550,102 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bleu clair</t>
+          <t>bleu</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>5c+</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>10</v>
+          <t>5a</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>noir</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>5c</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>6a</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>violet</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5a+</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>